<commit_message>
feat(ui): updated the table
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/apps/backend/excel-data/holidaystudentsub_library_migration.xlsx
+++ b/apps/backend/excel-data/holidaystudentsub_library_migration.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1981" uniqueCount="667">
   <si>
     <t>legacy_id</t>
   </si>
@@ -1670,6 +1670,348 @@
   </si>
   <si>
     <t>2026-06-20T07:51:52.367Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:51:53.703Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:51:55.160Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:51:56.709Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:51:58.299Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:51:59.602Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:00.980Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:02.072Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:03.597Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:05.186Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:06.825Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:09.054Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:10.605Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:12.741Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:14.070Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:15.425Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:16.945Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:18.506Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:20.092Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:22.140Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:23.707Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:26.019Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:29.795Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:32.160Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:34.325Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:37.425Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:40.211Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:41.924Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:43.386Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:45.219Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:46.647Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:47.845Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:49.616Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:51.191Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:52.683Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:54.003Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:55.548Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:57.080Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:52:59.045Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:00.822Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:02.223Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:03.435Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:04.714Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:06.613Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:08.256Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:09.591Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:11.014Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:12.171Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:13.400Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:15.118Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:16.433Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:17.570Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:18.692Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:19.832Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:21.197Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:22.276Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:23.303Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:24.369Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:25.434Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:26.498Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:27.709Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:28.724Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:29.687Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:30.650Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:32.193Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:33.465Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:34.515Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:35.587Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:36.791Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:37.822Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:39.308Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:40.384Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:41.965Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:43.356Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:44.796Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:46.411Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:47.876Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:49.217Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:50.663Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:52.661Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:54.409Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:55.852Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:57.339Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:53:59.035Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:00.545Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:01.916Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:03.027Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:04.575Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:05.998Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:07.521Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:08.868Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:10.119Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:11.414Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:12.490Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:13.832Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:15.387Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:16.838Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:18.238Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:19.563Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:20.998Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:22.595Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:23.968Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:25.458Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:26.778Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:28.316Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:29.581Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:30.860Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:32.127Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:33.863Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:35.383Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:36.626Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:37.926Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:39.267Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:40.844Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T07:54:41.873Z</t>
   </si>
 </sst>
 </file>
@@ -2050,7 +2392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D546"/>
+  <dimension ref="A1:D660"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -9697,6 +10039,1602 @@
         <v>552</v>
       </c>
     </row>
+    <row r="547" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A547">
+        <v>807</v>
+      </c>
+      <c r="B547" t="s">
+        <v>4</v>
+      </c>
+      <c r="C547" t="s">
+        <v>5</v>
+      </c>
+      <c r="D547" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="548" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A548">
+        <v>808</v>
+      </c>
+      <c r="B548" t="s">
+        <v>4</v>
+      </c>
+      <c r="C548" t="s">
+        <v>5</v>
+      </c>
+      <c r="D548" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="549" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A549">
+        <v>809</v>
+      </c>
+      <c r="B549" t="s">
+        <v>4</v>
+      </c>
+      <c r="C549" t="s">
+        <v>5</v>
+      </c>
+      <c r="D549" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="550" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A550">
+        <v>810</v>
+      </c>
+      <c r="B550" t="s">
+        <v>4</v>
+      </c>
+      <c r="C550" t="s">
+        <v>5</v>
+      </c>
+      <c r="D550" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="551" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A551">
+        <v>811</v>
+      </c>
+      <c r="B551" t="s">
+        <v>4</v>
+      </c>
+      <c r="C551" t="s">
+        <v>5</v>
+      </c>
+      <c r="D551" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="552" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A552">
+        <v>812</v>
+      </c>
+      <c r="B552" t="s">
+        <v>4</v>
+      </c>
+      <c r="C552" t="s">
+        <v>5</v>
+      </c>
+      <c r="D552" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="553" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A553">
+        <v>813</v>
+      </c>
+      <c r="B553" t="s">
+        <v>7</v>
+      </c>
+      <c r="C553" t="s">
+        <v>8</v>
+      </c>
+      <c r="D553" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="554" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A554">
+        <v>814</v>
+      </c>
+      <c r="B554" t="s">
+        <v>4</v>
+      </c>
+      <c r="C554" t="s">
+        <v>5</v>
+      </c>
+      <c r="D554" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="555" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A555">
+        <v>815</v>
+      </c>
+      <c r="B555" t="s">
+        <v>4</v>
+      </c>
+      <c r="C555" t="s">
+        <v>5</v>
+      </c>
+      <c r="D555" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="556" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A556">
+        <v>816</v>
+      </c>
+      <c r="B556" t="s">
+        <v>4</v>
+      </c>
+      <c r="C556" t="s">
+        <v>5</v>
+      </c>
+      <c r="D556" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="557" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A557">
+        <v>817</v>
+      </c>
+      <c r="B557" t="s">
+        <v>4</v>
+      </c>
+      <c r="C557" t="s">
+        <v>5</v>
+      </c>
+      <c r="D557" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="558" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A558">
+        <v>818</v>
+      </c>
+      <c r="B558" t="s">
+        <v>7</v>
+      </c>
+      <c r="C558" t="s">
+        <v>8</v>
+      </c>
+      <c r="D558" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="559" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A559">
+        <v>819</v>
+      </c>
+      <c r="B559" t="s">
+        <v>4</v>
+      </c>
+      <c r="C559" t="s">
+        <v>5</v>
+      </c>
+      <c r="D559" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="560" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A560">
+        <v>820</v>
+      </c>
+      <c r="B560" t="s">
+        <v>7</v>
+      </c>
+      <c r="C560" t="s">
+        <v>8</v>
+      </c>
+      <c r="D560" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="561" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A561">
+        <v>821</v>
+      </c>
+      <c r="B561" t="s">
+        <v>4</v>
+      </c>
+      <c r="C561" t="s">
+        <v>5</v>
+      </c>
+      <c r="D561" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="562" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A562">
+        <v>822</v>
+      </c>
+      <c r="B562" t="s">
+        <v>4</v>
+      </c>
+      <c r="C562" t="s">
+        <v>5</v>
+      </c>
+      <c r="D562" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="563" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A563">
+        <v>823</v>
+      </c>
+      <c r="B563" t="s">
+        <v>4</v>
+      </c>
+      <c r="C563" t="s">
+        <v>5</v>
+      </c>
+      <c r="D563" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="564" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A564">
+        <v>824</v>
+      </c>
+      <c r="B564" t="s">
+        <v>4</v>
+      </c>
+      <c r="C564" t="s">
+        <v>5</v>
+      </c>
+      <c r="D564" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="565" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A565">
+        <v>825</v>
+      </c>
+      <c r="B565" t="s">
+        <v>4</v>
+      </c>
+      <c r="C565" t="s">
+        <v>5</v>
+      </c>
+      <c r="D565" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="566" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A566">
+        <v>826</v>
+      </c>
+      <c r="B566" t="s">
+        <v>4</v>
+      </c>
+      <c r="C566" t="s">
+        <v>5</v>
+      </c>
+      <c r="D566" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="567" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A567">
+        <v>827</v>
+      </c>
+      <c r="B567" t="s">
+        <v>4</v>
+      </c>
+      <c r="C567" t="s">
+        <v>5</v>
+      </c>
+      <c r="D567" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="568" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A568">
+        <v>828</v>
+      </c>
+      <c r="B568" t="s">
+        <v>4</v>
+      </c>
+      <c r="C568" t="s">
+        <v>5</v>
+      </c>
+      <c r="D568" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="569" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A569">
+        <v>829</v>
+      </c>
+      <c r="B569" t="s">
+        <v>4</v>
+      </c>
+      <c r="C569" t="s">
+        <v>5</v>
+      </c>
+      <c r="D569" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="570" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A570">
+        <v>830</v>
+      </c>
+      <c r="B570" t="s">
+        <v>4</v>
+      </c>
+      <c r="C570" t="s">
+        <v>5</v>
+      </c>
+      <c r="D570" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="571" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A571">
+        <v>831</v>
+      </c>
+      <c r="B571" t="s">
+        <v>4</v>
+      </c>
+      <c r="C571" t="s">
+        <v>5</v>
+      </c>
+      <c r="D571" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="572" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A572">
+        <v>832</v>
+      </c>
+      <c r="B572" t="s">
+        <v>4</v>
+      </c>
+      <c r="C572" t="s">
+        <v>5</v>
+      </c>
+      <c r="D572" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="573" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A573">
+        <v>833</v>
+      </c>
+      <c r="B573" t="s">
+        <v>4</v>
+      </c>
+      <c r="C573" t="s">
+        <v>5</v>
+      </c>
+      <c r="D573" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="574" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A574">
+        <v>834</v>
+      </c>
+      <c r="B574" t="s">
+        <v>4</v>
+      </c>
+      <c r="C574" t="s">
+        <v>5</v>
+      </c>
+      <c r="D574" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="575" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A575">
+        <v>835</v>
+      </c>
+      <c r="B575" t="s">
+        <v>4</v>
+      </c>
+      <c r="C575" t="s">
+        <v>5</v>
+      </c>
+      <c r="D575" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="576" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A576">
+        <v>836</v>
+      </c>
+      <c r="B576" t="s">
+        <v>4</v>
+      </c>
+      <c r="C576" t="s">
+        <v>5</v>
+      </c>
+      <c r="D576" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="577" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A577">
+        <v>837</v>
+      </c>
+      <c r="B577" t="s">
+        <v>7</v>
+      </c>
+      <c r="C577" t="s">
+        <v>8</v>
+      </c>
+      <c r="D577" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="578" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A578">
+        <v>838</v>
+      </c>
+      <c r="B578" t="s">
+        <v>4</v>
+      </c>
+      <c r="C578" t="s">
+        <v>5</v>
+      </c>
+      <c r="D578" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="579" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A579">
+        <v>839</v>
+      </c>
+      <c r="B579" t="s">
+        <v>7</v>
+      </c>
+      <c r="C579" t="s">
+        <v>8</v>
+      </c>
+      <c r="D579" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="580" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A580">
+        <v>840</v>
+      </c>
+      <c r="B580" t="s">
+        <v>4</v>
+      </c>
+      <c r="C580" t="s">
+        <v>5</v>
+      </c>
+      <c r="D580" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="581" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A581">
+        <v>841</v>
+      </c>
+      <c r="B581" t="s">
+        <v>4</v>
+      </c>
+      <c r="C581" t="s">
+        <v>5</v>
+      </c>
+      <c r="D581" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="582" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A582">
+        <v>842</v>
+      </c>
+      <c r="B582" t="s">
+        <v>4</v>
+      </c>
+      <c r="C582" t="s">
+        <v>5</v>
+      </c>
+      <c r="D582" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="583" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A583">
+        <v>843</v>
+      </c>
+      <c r="B583" t="s">
+        <v>4</v>
+      </c>
+      <c r="C583" t="s">
+        <v>5</v>
+      </c>
+      <c r="D583" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="584" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A584">
+        <v>844</v>
+      </c>
+      <c r="B584" t="s">
+        <v>7</v>
+      </c>
+      <c r="C584" t="s">
+        <v>8</v>
+      </c>
+      <c r="D584" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="585" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A585">
+        <v>845</v>
+      </c>
+      <c r="B585" t="s">
+        <v>7</v>
+      </c>
+      <c r="C585" t="s">
+        <v>8</v>
+      </c>
+      <c r="D585" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="586" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A586">
+        <v>846</v>
+      </c>
+      <c r="B586" t="s">
+        <v>7</v>
+      </c>
+      <c r="C586" t="s">
+        <v>8</v>
+      </c>
+      <c r="D586" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="587" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A587">
+        <v>847</v>
+      </c>
+      <c r="B587" t="s">
+        <v>7</v>
+      </c>
+      <c r="C587" t="s">
+        <v>8</v>
+      </c>
+      <c r="D587" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="588" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A588">
+        <v>848</v>
+      </c>
+      <c r="B588" t="s">
+        <v>7</v>
+      </c>
+      <c r="C588" t="s">
+        <v>8</v>
+      </c>
+      <c r="D588" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="589" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A589">
+        <v>849</v>
+      </c>
+      <c r="B589" t="s">
+        <v>7</v>
+      </c>
+      <c r="C589" t="s">
+        <v>8</v>
+      </c>
+      <c r="D589" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="590" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A590">
+        <v>850</v>
+      </c>
+      <c r="B590" t="s">
+        <v>7</v>
+      </c>
+      <c r="C590" t="s">
+        <v>8</v>
+      </c>
+      <c r="D590" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="591" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A591">
+        <v>851</v>
+      </c>
+      <c r="B591" t="s">
+        <v>7</v>
+      </c>
+      <c r="C591" t="s">
+        <v>8</v>
+      </c>
+      <c r="D591" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="592" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A592">
+        <v>852</v>
+      </c>
+      <c r="B592" t="s">
+        <v>7</v>
+      </c>
+      <c r="C592" t="s">
+        <v>8</v>
+      </c>
+      <c r="D592" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="593" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A593">
+        <v>853</v>
+      </c>
+      <c r="B593" t="s">
+        <v>7</v>
+      </c>
+      <c r="C593" t="s">
+        <v>8</v>
+      </c>
+      <c r="D593" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="594" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A594">
+        <v>854</v>
+      </c>
+      <c r="B594" t="s">
+        <v>7</v>
+      </c>
+      <c r="C594" t="s">
+        <v>8</v>
+      </c>
+      <c r="D594" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="595" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A595">
+        <v>855</v>
+      </c>
+      <c r="B595" t="s">
+        <v>7</v>
+      </c>
+      <c r="C595" t="s">
+        <v>8</v>
+      </c>
+      <c r="D595" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="596" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A596">
+        <v>856</v>
+      </c>
+      <c r="B596" t="s">
+        <v>7</v>
+      </c>
+      <c r="C596" t="s">
+        <v>8</v>
+      </c>
+      <c r="D596" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="597" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A597">
+        <v>857</v>
+      </c>
+      <c r="B597" t="s">
+        <v>7</v>
+      </c>
+      <c r="C597" t="s">
+        <v>8</v>
+      </c>
+      <c r="D597" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="598" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A598">
+        <v>858</v>
+      </c>
+      <c r="B598" t="s">
+        <v>7</v>
+      </c>
+      <c r="C598" t="s">
+        <v>8</v>
+      </c>
+      <c r="D598" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="599" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A599">
+        <v>859</v>
+      </c>
+      <c r="B599" t="s">
+        <v>7</v>
+      </c>
+      <c r="C599" t="s">
+        <v>8</v>
+      </c>
+      <c r="D599" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="600" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A600">
+        <v>860</v>
+      </c>
+      <c r="B600" t="s">
+        <v>7</v>
+      </c>
+      <c r="C600" t="s">
+        <v>8</v>
+      </c>
+      <c r="D600" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="601" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A601">
+        <v>861</v>
+      </c>
+      <c r="B601" t="s">
+        <v>7</v>
+      </c>
+      <c r="C601" t="s">
+        <v>8</v>
+      </c>
+      <c r="D601" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="602" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A602">
+        <v>862</v>
+      </c>
+      <c r="B602" t="s">
+        <v>7</v>
+      </c>
+      <c r="C602" t="s">
+        <v>8</v>
+      </c>
+      <c r="D602" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="603" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A603">
+        <v>863</v>
+      </c>
+      <c r="B603" t="s">
+        <v>7</v>
+      </c>
+      <c r="C603" t="s">
+        <v>8</v>
+      </c>
+      <c r="D603" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="604" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A604">
+        <v>864</v>
+      </c>
+      <c r="B604" t="s">
+        <v>7</v>
+      </c>
+      <c r="C604" t="s">
+        <v>8</v>
+      </c>
+      <c r="D604" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="605" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A605">
+        <v>865</v>
+      </c>
+      <c r="B605" t="s">
+        <v>7</v>
+      </c>
+      <c r="C605" t="s">
+        <v>8</v>
+      </c>
+      <c r="D605" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="606" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A606">
+        <v>866</v>
+      </c>
+      <c r="B606" t="s">
+        <v>7</v>
+      </c>
+      <c r="C606" t="s">
+        <v>8</v>
+      </c>
+      <c r="D606" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="607" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A607">
+        <v>867</v>
+      </c>
+      <c r="B607" t="s">
+        <v>7</v>
+      </c>
+      <c r="C607" t="s">
+        <v>8</v>
+      </c>
+      <c r="D607" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="608" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A608">
+        <v>868</v>
+      </c>
+      <c r="B608" t="s">
+        <v>7</v>
+      </c>
+      <c r="C608" t="s">
+        <v>8</v>
+      </c>
+      <c r="D608" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="609" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A609">
+        <v>869</v>
+      </c>
+      <c r="B609" t="s">
+        <v>7</v>
+      </c>
+      <c r="C609" t="s">
+        <v>8</v>
+      </c>
+      <c r="D609" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="610" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A610">
+        <v>870</v>
+      </c>
+      <c r="B610" t="s">
+        <v>7</v>
+      </c>
+      <c r="C610" t="s">
+        <v>8</v>
+      </c>
+      <c r="D610" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="611" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A611">
+        <v>871</v>
+      </c>
+      <c r="B611" t="s">
+        <v>7</v>
+      </c>
+      <c r="C611" t="s">
+        <v>8</v>
+      </c>
+      <c r="D611" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="612" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A612">
+        <v>872</v>
+      </c>
+      <c r="B612" t="s">
+        <v>7</v>
+      </c>
+      <c r="C612" t="s">
+        <v>8</v>
+      </c>
+      <c r="D612" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="613" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A613">
+        <v>873</v>
+      </c>
+      <c r="B613" t="s">
+        <v>7</v>
+      </c>
+      <c r="C613" t="s">
+        <v>8</v>
+      </c>
+      <c r="D613" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="614" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A614">
+        <v>874</v>
+      </c>
+      <c r="B614" t="s">
+        <v>7</v>
+      </c>
+      <c r="C614" t="s">
+        <v>8</v>
+      </c>
+      <c r="D614" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="615" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A615">
+        <v>875</v>
+      </c>
+      <c r="B615" t="s">
+        <v>7</v>
+      </c>
+      <c r="C615" t="s">
+        <v>8</v>
+      </c>
+      <c r="D615" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="616" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A616">
+        <v>876</v>
+      </c>
+      <c r="B616" t="s">
+        <v>4</v>
+      </c>
+      <c r="C616" t="s">
+        <v>5</v>
+      </c>
+      <c r="D616" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="617" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A617">
+        <v>877</v>
+      </c>
+      <c r="B617" t="s">
+        <v>7</v>
+      </c>
+      <c r="C617" t="s">
+        <v>8</v>
+      </c>
+      <c r="D617" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="618" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A618">
+        <v>878</v>
+      </c>
+      <c r="B618" t="s">
+        <v>4</v>
+      </c>
+      <c r="C618" t="s">
+        <v>5</v>
+      </c>
+      <c r="D618" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="619" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A619">
+        <v>879</v>
+      </c>
+      <c r="B619" t="s">
+        <v>4</v>
+      </c>
+      <c r="C619" t="s">
+        <v>5</v>
+      </c>
+      <c r="D619" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="620" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A620">
+        <v>880</v>
+      </c>
+      <c r="B620" t="s">
+        <v>4</v>
+      </c>
+      <c r="C620" t="s">
+        <v>5</v>
+      </c>
+      <c r="D620" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="621" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A621">
+        <v>881</v>
+      </c>
+      <c r="B621" t="s">
+        <v>4</v>
+      </c>
+      <c r="C621" t="s">
+        <v>5</v>
+      </c>
+      <c r="D621" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="622" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A622">
+        <v>882</v>
+      </c>
+      <c r="B622" t="s">
+        <v>4</v>
+      </c>
+      <c r="C622" t="s">
+        <v>5</v>
+      </c>
+      <c r="D622" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="623" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A623">
+        <v>883</v>
+      </c>
+      <c r="B623" t="s">
+        <v>4</v>
+      </c>
+      <c r="C623" t="s">
+        <v>5</v>
+      </c>
+      <c r="D623" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="624" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A624">
+        <v>884</v>
+      </c>
+      <c r="B624" t="s">
+        <v>4</v>
+      </c>
+      <c r="C624" t="s">
+        <v>5</v>
+      </c>
+      <c r="D624" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="625" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A625">
+        <v>885</v>
+      </c>
+      <c r="B625" t="s">
+        <v>4</v>
+      </c>
+      <c r="C625" t="s">
+        <v>5</v>
+      </c>
+      <c r="D625" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="626" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A626">
+        <v>886</v>
+      </c>
+      <c r="B626" t="s">
+        <v>4</v>
+      </c>
+      <c r="C626" t="s">
+        <v>5</v>
+      </c>
+      <c r="D626" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="627" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A627">
+        <v>887</v>
+      </c>
+      <c r="B627" t="s">
+        <v>4</v>
+      </c>
+      <c r="C627" t="s">
+        <v>5</v>
+      </c>
+      <c r="D627" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="628" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A628">
+        <v>888</v>
+      </c>
+      <c r="B628" t="s">
+        <v>4</v>
+      </c>
+      <c r="C628" t="s">
+        <v>5</v>
+      </c>
+      <c r="D628" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="629" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A629">
+        <v>889</v>
+      </c>
+      <c r="B629" t="s">
+        <v>4</v>
+      </c>
+      <c r="C629" t="s">
+        <v>5</v>
+      </c>
+      <c r="D629" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="630" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A630">
+        <v>890</v>
+      </c>
+      <c r="B630" t="s">
+        <v>4</v>
+      </c>
+      <c r="C630" t="s">
+        <v>5</v>
+      </c>
+      <c r="D630" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="631" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A631">
+        <v>891</v>
+      </c>
+      <c r="B631" t="s">
+        <v>4</v>
+      </c>
+      <c r="C631" t="s">
+        <v>5</v>
+      </c>
+      <c r="D631" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="632" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A632">
+        <v>892</v>
+      </c>
+      <c r="B632" t="s">
+        <v>7</v>
+      </c>
+      <c r="C632" t="s">
+        <v>8</v>
+      </c>
+      <c r="D632" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="633" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A633">
+        <v>893</v>
+      </c>
+      <c r="B633" t="s">
+        <v>4</v>
+      </c>
+      <c r="C633" t="s">
+        <v>5</v>
+      </c>
+      <c r="D633" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="634" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A634">
+        <v>894</v>
+      </c>
+      <c r="B634" t="s">
+        <v>4</v>
+      </c>
+      <c r="C634" t="s">
+        <v>5</v>
+      </c>
+      <c r="D634" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="635" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A635">
+        <v>895</v>
+      </c>
+      <c r="B635" t="s">
+        <v>4</v>
+      </c>
+      <c r="C635" t="s">
+        <v>5</v>
+      </c>
+      <c r="D635" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="636" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A636">
+        <v>896</v>
+      </c>
+      <c r="B636" t="s">
+        <v>4</v>
+      </c>
+      <c r="C636" t="s">
+        <v>5</v>
+      </c>
+      <c r="D636" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="637" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A637">
+        <v>897</v>
+      </c>
+      <c r="B637" t="s">
+        <v>7</v>
+      </c>
+      <c r="C637" t="s">
+        <v>8</v>
+      </c>
+      <c r="D637" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="638" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A638">
+        <v>898</v>
+      </c>
+      <c r="B638" t="s">
+        <v>4</v>
+      </c>
+      <c r="C638" t="s">
+        <v>5</v>
+      </c>
+      <c r="D638" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="639" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A639">
+        <v>899</v>
+      </c>
+      <c r="B639" t="s">
+        <v>7</v>
+      </c>
+      <c r="C639" t="s">
+        <v>8</v>
+      </c>
+      <c r="D639" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="640" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A640">
+        <v>900</v>
+      </c>
+      <c r="B640" t="s">
+        <v>4</v>
+      </c>
+      <c r="C640" t="s">
+        <v>5</v>
+      </c>
+      <c r="D640" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="641" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A641">
+        <v>901</v>
+      </c>
+      <c r="B641" t="s">
+        <v>4</v>
+      </c>
+      <c r="C641" t="s">
+        <v>5</v>
+      </c>
+      <c r="D641" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="642" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A642">
+        <v>902</v>
+      </c>
+      <c r="B642" t="s">
+        <v>4</v>
+      </c>
+      <c r="C642" t="s">
+        <v>5</v>
+      </c>
+      <c r="D642" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="643" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A643">
+        <v>903</v>
+      </c>
+      <c r="B643" t="s">
+        <v>4</v>
+      </c>
+      <c r="C643" t="s">
+        <v>5</v>
+      </c>
+      <c r="D643" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="644" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A644">
+        <v>904</v>
+      </c>
+      <c r="B644" t="s">
+        <v>4</v>
+      </c>
+      <c r="C644" t="s">
+        <v>5</v>
+      </c>
+      <c r="D644" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="645" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A645">
+        <v>905</v>
+      </c>
+      <c r="B645" t="s">
+        <v>4</v>
+      </c>
+      <c r="C645" t="s">
+        <v>5</v>
+      </c>
+      <c r="D645" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="646" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A646">
+        <v>906</v>
+      </c>
+      <c r="B646" t="s">
+        <v>4</v>
+      </c>
+      <c r="C646" t="s">
+        <v>5</v>
+      </c>
+      <c r="D646" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="647" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A647">
+        <v>907</v>
+      </c>
+      <c r="B647" t="s">
+        <v>4</v>
+      </c>
+      <c r="C647" t="s">
+        <v>5</v>
+      </c>
+      <c r="D647" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="648" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A648">
+        <v>908</v>
+      </c>
+      <c r="B648" t="s">
+        <v>4</v>
+      </c>
+      <c r="C648" t="s">
+        <v>5</v>
+      </c>
+      <c r="D648" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="649" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A649">
+        <v>909</v>
+      </c>
+      <c r="B649" t="s">
+        <v>4</v>
+      </c>
+      <c r="C649" t="s">
+        <v>5</v>
+      </c>
+      <c r="D649" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="650" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A650">
+        <v>910</v>
+      </c>
+      <c r="B650" t="s">
+        <v>4</v>
+      </c>
+      <c r="C650" t="s">
+        <v>5</v>
+      </c>
+      <c r="D650" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="651" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A651">
+        <v>911</v>
+      </c>
+      <c r="B651" t="s">
+        <v>4</v>
+      </c>
+      <c r="C651" t="s">
+        <v>5</v>
+      </c>
+      <c r="D651" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="652" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A652">
+        <v>912</v>
+      </c>
+      <c r="B652" t="s">
+        <v>4</v>
+      </c>
+      <c r="C652" t="s">
+        <v>5</v>
+      </c>
+      <c r="D652" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="653" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A653">
+        <v>913</v>
+      </c>
+      <c r="B653" t="s">
+        <v>4</v>
+      </c>
+      <c r="C653" t="s">
+        <v>5</v>
+      </c>
+      <c r="D653" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="654" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A654">
+        <v>914</v>
+      </c>
+      <c r="B654" t="s">
+        <v>4</v>
+      </c>
+      <c r="C654" t="s">
+        <v>5</v>
+      </c>
+      <c r="D654" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="655" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A655">
+        <v>915</v>
+      </c>
+      <c r="B655" t="s">
+        <v>4</v>
+      </c>
+      <c r="C655" t="s">
+        <v>5</v>
+      </c>
+      <c r="D655" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="656" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A656">
+        <v>916</v>
+      </c>
+      <c r="B656" t="s">
+        <v>4</v>
+      </c>
+      <c r="C656" t="s">
+        <v>5</v>
+      </c>
+      <c r="D656" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="657" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A657">
+        <v>917</v>
+      </c>
+      <c r="B657" t="s">
+        <v>4</v>
+      </c>
+      <c r="C657" t="s">
+        <v>5</v>
+      </c>
+      <c r="D657" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="658" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A658">
+        <v>918</v>
+      </c>
+      <c r="B658" t="s">
+        <v>4</v>
+      </c>
+      <c r="C658" t="s">
+        <v>5</v>
+      </c>
+      <c r="D658" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="659" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A659">
+        <v>919</v>
+      </c>
+      <c r="B659" t="s">
+        <v>4</v>
+      </c>
+      <c r="C659" t="s">
+        <v>5</v>
+      </c>
+      <c r="D659" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="660" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A660">
+        <v>920</v>
+      </c>
+      <c r="B660" t="s">
+        <v>7</v>
+      </c>
+      <c r="C660" t="s">
+        <v>8</v>
+      </c>
+      <c r="D660" t="s">
+        <v>666</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>